<commit_message>
feat: add seat detail panel
</commit_message>
<xml_diff>
--- a/data/layouts/minowa_uno_coordinate_map.xlsx
+++ b/data/layouts/minowa_uno_coordinate_map.xlsx
@@ -5,12 +5,12 @@
   <workbookPr/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
-      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\terry\Downloads\"/>
+      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\terry\MUP\GitHub\mup\data\layouts\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{C53035FA-1C2D-4DB8-AA22-8022C41F6FC2}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{7A6A7D28-B206-42F8-8087-2F7EC0AA965C}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="2190" yWindow="480" windowWidth="23655" windowHeight="14460" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="1170" yWindow="1170" windowWidth="23655" windowHeight="14460" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="座標マップ" sheetId="1" r:id="rId1"/>
@@ -1594,7 +1594,7 @@
         <v>641</v>
       </c>
       <c r="S13" s="2">
-        <v>42</v>
+        <v>642</v>
       </c>
       <c r="T13" s="2">
         <v>643</v>

</xml_diff>